<commit_message>
voice demo changed new
</commit_message>
<xml_diff>
--- a/data/call-qualifications.xlsx
+++ b/data/call-qualifications.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:R21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,10 +460,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-04-28T08:12:20.478Z</v>
+        <v>2026-04-28T10:09:01.826Z</v>
       </c>
       <c r="C2" t="str">
-        <v>+919328481970</v>
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -478,7 +478,7 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I2" t="str">
         <v>Gujarati</v>
@@ -499,15 +499,592 @@
         <v>unknown</v>
       </c>
       <c r="O2" t="str">
+        <v>ના.</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>conv_9101kq9rx3nbf3hsqrspc9b7zk5q</v>
+      </c>
+      <c r="R2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be...
+Prospect: Gujarati.
+Agent: સ્વાગત છે.શું તમે મા ઉમિયા અને વિશ્વ ઉમિયા ફાઉન્ડેશન વિશે સંક્ષિપ્ત સંદેશ સાંભળવા માંગો છો?
+Prospect: હા।
+Agent: ધન્યવાદ. ઉમિયા ધામ વિશ્વના સૌથી ઊંચા મંદિરોમાંના એક તરીકે વિકસાવવામાં આવી રહ્યું છે, જે ભક્તિ, એકતા અને આસ્થાનું પ્રતીક છે.વિશ્વ ઉમિયા ફાઉન્ડેશન આધ્યાત્મિકતા, શિક્ષણ, સ્વાસ્થ્ય અને સમુદાયની ઉન્નતિ દ્વારા સમાજની સેવા કરે છે.કેમ કે તમે વધુ જાણવા માંગો છો કે અમારી ટીમ સાથે જોડાવા માંગો છો?
+Prospect: હમ, વધુ જાણવા માંગીએ છીએ.હમ, વધુ જાણવા માંગીએ છીએ.
+Agent: સરસ! વિશ્વ ઉમિયા ફાઉન્ડેશન આધ્યાત્મિકતા, શિક્ષણ, સ્વાસ્થ્ય અને સમુદાયની ઉન્નતિ દ્વારા સમાજની સેવા કરે છે. ઉમિયા ધામ વિશ્વના સૌથી ઊંચા મંદિરોમાંના એક તરીકે વિકસાવવામાં આવી રહ્યું છે, જે ભક્તિ, એકતા અને આસ્થાનું પ્રતીક છે. વધુ માહિતી માટે આપણી વેબસાઇટ પર જોવા માટે આવો: https://www.vuf.org/ કે અમારી ટીમ સાથે જોડાવા માંગો છો?
+Prospect: ના.
+Agent: ...</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-04-28T10:06:59.684Z</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>5</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Hindi</v>
+      </c>
+      <c r="J3" t="str">
+        <v>hi</v>
+      </c>
+      <c r="K3" t="str">
+        <v>English, Hindi</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N3" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O3" t="str">
+        <v>हाँ, मैं अधिक जानना चाहूंगा।</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>conv_7601kq9rv4d2e9rrjrjwdbm3b48p</v>
+      </c>
+      <c r="R3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief messa...
+Prospect: Hindi.
+Agent: धन्यवाद।उमिया धाम विश्व के सबसे ऊंचे मंदिरों में से एक के रूप में विकसित किया जा रहा है, जो आस्था, एकता और भक्ति का प्रतीक है।विश्व उमिया फाउंडेशन स्पिरिचुअलिटी, शिक्षा, स्वास्थ्य और समुदाय उन्नयन के माध्यम से समाज की सेवा करता है।क्या आप अधिक जानना चाहेंगे या हमारी टीम से जुड़ना चाहेंगे?
+Prospect: हाँ, मैं अधिक जानना चाहूंगा।
+Agent: [excited] बहुत अच्छा! आप वेबसाइट पर अधिक जानकारी प्राप्त कर सकते हैं: https://www.vuf.org/क्या आप अपने...</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-04-28T10:01:48.637Z</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>7</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Gujarati</v>
+      </c>
+      <c r="J4" t="str">
+        <v>gu</v>
+      </c>
+      <c r="K4" t="str">
+        <v>English, Gujarati</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N4" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O4" t="str">
+        <v>હા।</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>conv_5701kq9rh34nfy9s02fpz6mb9cng</v>
+      </c>
+      <c r="R4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a ...
+Prospect: Gujarat.
+Agent: સ્વાગત છે!કૃપા કરીને જણાવો કે તમે કયા ભાષામાં વાત કરવામાં આરામદાયક માનો છો — અંગ્રેજી, હિન્દી, કે ગુજરાતી?
+Prospect: ગુજરાતી.
+Agent: સ્વાગત છે!અમારી સેવાઓ વિશે થોડો સમય લઈને સાંભળવા તમારી સાથે વાત કરવા તમારી તૈયારી છે?
+Prospect: હા।
+Agent: ધન્યવાદ. ઉમિયા ધામ વિશ્વના સૌથી ઊંચા મંદિરોમાંના એક તરીકે વિકસાવવામાં આવી રહ્યું છે, જે ભક્તિ, એકતા અને આધ્યાત્મિકતાનું પ્રતીક છે.વિશ્વ ઉમિયા ફાઉન્ડેશન આધ્યાત્મિકતા, શિક્ષણ, સ્વાસ્થ્ય અને સમાજની ઉન્નતિ દ્વારા સમાજની સેવા કરે છે.કેમ કે તમને વધુ જાણવા માંગો છો કે અમારી ટીમ સાથે જોડાવા માંગો છો?</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-04-28T09:49:46.217Z</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>5</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Gujarati</v>
+      </c>
+      <c r="J5" t="str">
+        <v>gu</v>
+      </c>
+      <c r="K5" t="str">
+        <v>English, Gujarati</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N5" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O5" t="str">
+        <v>...</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>conv_2601kq9qvs1jebds4t54m74mvpkt</v>
+      </c>
+      <c r="R5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear...
+Prospect: હિન્દુ.
+Agent: સારું છે, હું હિન્દીમાં વાત કરીશ।કૃપા કરીને જણાવો કે કેટલો સમય તમને લાગે છે?[slow] મેં તમને માતા ઉમિયા અને વિશ્વ ઉમિયા ફાઉન્ડેશન વિશે થોડી માહિતી આપવા માંગુ છું।
+Prospect: ...
+Agent: કૃપા કરીને જણાવો, કે કેટલો સમય તમને લાગે છે?[slow] મેં તમને માતા ઉમિયા અને વિશ્વ ઉમિયા ફાઉન્ડેશન વિશે થોડી માહિતી આપવા માંગુ છું।...</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-04-28T09:43:59.661Z</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="str">
+        <v>English</v>
+      </c>
+      <c r="J6" t="str">
+        <v>en</v>
+      </c>
+      <c r="K6" t="str">
+        <v>English</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N6" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief message about Maa Umiya and our mission?
+Umiya Dham is being develope</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>conv_3701kq9qgpj7fx5vbjnb0k742b1d</v>
+      </c>
+      <c r="R6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief message about Maa Umiya and our mission?
+Umiya Dham is being developed as one of the tallest temples in the world, symbolizing strength, devotion, and cultural pride, and spreading a message of unity and spirituality.
+At Vishv Umiya Foundation, the mission is to uplift society through spirituality, education, healthcare, and community service, creating a better and brighter future for all.
+"Thank you for connecting with Vishv Umiya Foundation. We truly value your time. May Maa Umiya bless you and your family. Have a wonderful day...</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-04-28T09:43:34.372Z</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>5</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Gujarati</v>
+      </c>
+      <c r="J7" t="str">
+        <v>gu</v>
+      </c>
+      <c r="K7" t="str">
+        <v>English, Gujarati</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N7" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O7" t="str">
+        <v>...</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>conv_3201kq9qgyvae3sby1cd2k9d91wx</v>
+      </c>
+      <c r="R7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief message about Maa Umiya and our mission?
+Umiya Dham is being developed as one of...
+Prospect: હાં.
+Agent: [happy] ધન્યવાદ! કૃપા કરીને કહો કે તમે કયા ભાષામાં સુવિધા માટે આરામથી બોલવા માંગો છો — અંગ્રેજી, હિન્દી કે ગુજરાતી?
+Prospect: ...
+Agent: [soft] હું સમજું...</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-04-28T09:41:51.754Z</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>7</v>
+      </c>
+      <c r="I8" t="str">
+        <v>English</v>
+      </c>
+      <c r="J8" t="str">
+        <v>en</v>
+      </c>
+      <c r="K8" t="str">
+        <v>English, Gujarati</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N8" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Thank you.</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>conv_9401kq9qd86qea2rg6xtnzj9fw5s</v>
+      </c>
+      <c r="R8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing ...
+Prospect: નહીં.
+Agent: Thank you for your time. Maa Umiya bless you and your family. Have a peaceful day. Jai Maa Umiya 🙏
+Prospect: શું? તમને શું લાગે છે?તમને શું લાગે છે?તમે બોલવાનું જ ચાલુ કરો છો. હમ્મ.તમે બોલવાનું જ ચાલુ કરો છ
+Agent: ...
+Prospect: Thank you.
+Agent: You're welcome. May Maa Umiya bless you and your family. Have a wonderful da...</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-04-28T09:40:49.805Z</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9" t="str">
+        <v>English</v>
+      </c>
+      <c r="J9" t="str">
+        <v>en</v>
+      </c>
+      <c r="K9" t="str">
+        <v>English</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N9" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Hello?</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>conv_3701kq9qc50jf66b0kyccx2f2687</v>
+      </c>
+      <c r="R9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief message about Maa Umiya and our mission?
+Umiya Dham is being developed as one of the tallest temples in the world, symbolizing strength, devotion, a...
+Prospect: Hello?
+Agent: Hello, I'm here.Would you be willing to hear a brief message about Maa Umiya and Vishv Umiya Foundation?</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-04-28T09:40:25.307Z</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>11</v>
+      </c>
+      <c r="I10" t="str">
+        <v>English</v>
+      </c>
+      <c r="J10" t="str">
+        <v>en</v>
+      </c>
+      <c r="K10" t="str">
+        <v>English, Hindi, Gujarati</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Willing to join</v>
+      </c>
+      <c r="N10" t="str">
+        <v>willing_to_join</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Yes.</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>conv_9701kq9q8j4yftes3c09h4h0z6hs</v>
+      </c>
+      <c r="R10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Agent: Namaste 
+I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
+Would you be willing to hear a brief message about Maa Umiya and our mission?
+Umiya Dham is being developed as one of the tallest temples in the world, symbolizing strength, devotion, and cultural pride, and spreading a message of unity and spirituality.
+At Vishv Umiya Foundation, the mission is to uplift society through spirituality, education, healthcare, and community service, creating a better and brighter future for all.
+"Thank you for connecting with Vishv Umiya Foundation. We truly value your time. May Maa Umiya bless you and you...
+Prospect: PC अभी तो यही है।अच्छा।
+Agent: [slow] Thank you for your response.Would you like to know more about Umiya Dham and how the foundation is serving society through faith and service?
+Prospect: શું જરા થી?થોડું થોડું.
+Agent: [soft] Thank you for sharing. Would you like to know how Umiya Dham is being built as a symbol of devotion and unity, and how the Vishv Umiya Foundation supports education, healthcare, and community upliftment?
+Prospect: Yes.
+Agent: [calm] Umiya Dham is being developed as one of the tallest temples in the world, representing faith, unity, and spiritual strength.The Vishv Umiya Foundation serves society through education, healthcare, and community programs, spreading love and service.Would you like to visit our website to learn more? It’s https://www.vuf.org/
+Prospect: Yes.
+Agent: [gentle] Wonderful I’m glad you’re interested. You can visit our website at https://www.vuf.org/ to explore more about Umiya Dham and the foundation’s work.Would you like me to connect you with our team for further details?
+Prospect: Yes.
+Agent: [pleasant] Wonderful I’ll connect you with our team right away. Thank you for your time and interest in Vishv Umiya Foundation. May Maa Umiya bless you and your family. Have a wonderful day. Jai Maa Umiya 🙏</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-04-28T08:12:20.478Z</v>
+      </c>
+      <c r="C11" t="str">
+        <v>+919328481970</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>7</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Gujarati</v>
+      </c>
+      <c r="J11" t="str">
+        <v>gu</v>
+      </c>
+      <c r="K11" t="str">
+        <v>English, Gujarati</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N11" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="O11" t="str">
         <v>હા, મારે વધારે જાણવું છે વિશ્વ ઓમિયા foundation ના વિશે.</v>
       </c>
-      <c r="P2" t="str">
+      <c r="P11" t="str">
         <v>CA73824daf7f18e54de49c0bfa20f48f46</v>
       </c>
-      <c r="Q2" t="str">
+      <c r="Q11" t="str">
         <v>conv_6801kq9j82gce5087xcrta8mq6y4</v>
       </c>
-      <c r="R2" t="str" xml:space="preserve">
+      <c r="R11" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya a...
@@ -519,59 +1096,59 @@
 Agent: [calm] આભાર, તમારો રસ માટે ખુબ ખુબ આભાર. વિશ્વ ઉમિયા ફાઉન્ડેશન અમદાવાદમાં આધ્યાત્મિકતા, શિક્ષણ, સ્વાસ્થ્ય અને સમુદાય ઉન્નતિ માટ...</v>
       </c>
     </row>
-    <row r="3" xml:space="preserve">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
+    <row r="12" xml:space="preserve">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
         <v>2026-04-28T08:09:58.868Z</v>
       </c>
-      <c r="C3" t="str">
-        <v/>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v/>
-      </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
         <v>11</v>
       </c>
-      <c r="I3" t="str">
+      <c r="I12" t="str">
         <v>Gujarati</v>
       </c>
-      <c r="J3" t="str">
+      <c r="J12" t="str">
         <v>gu</v>
       </c>
-      <c r="K3" t="str">
+      <c r="K12" t="str">
         <v>English, Gujarati</v>
       </c>
-      <c r="L3" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="L12" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N12" t="str">
         <v>unknown</v>
       </c>
-      <c r="O3" t="str">
+      <c r="O12" t="str">
         <v>જય મા ઉમિયા.</v>
       </c>
-      <c r="P3" t="str">
-        <v/>
-      </c>
-      <c r="Q3" t="str">
+      <c r="P12" t="str">
+        <v/>
+      </c>
+      <c r="Q12" t="str">
         <v>conv_5801kq9j2ptef53sdz089y7qarx1</v>
       </c>
-      <c r="R3" t="str" xml:space="preserve">
+      <c r="R12" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -589,59 +1166,59 @@
 Agent: જય મા ઉમિયા! મા ઉમિયા તમને અને તમારા પરિવારને સદા આશીર્વાદ આપે. શુભ દિવસ રહે...</v>
       </c>
     </row>
-    <row r="4" xml:space="preserve">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
+    <row r="13" xml:space="preserve">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
         <v>2026-04-28T08:08:49.302Z</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
-      </c>
-      <c r="D4" t="str">
-        <v/>
-      </c>
-      <c r="E4" t="str">
-        <v/>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
         <v>5</v>
       </c>
-      <c r="I4" t="str">
+      <c r="I13" t="str">
         <v>Gujarati</v>
       </c>
-      <c r="J4" t="str">
+      <c r="J13" t="str">
         <v>gu</v>
       </c>
-      <c r="K4" t="str">
+      <c r="K13" t="str">
         <v>English, Gujarati</v>
       </c>
-      <c r="L4" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N4" t="str">
+      <c r="L13" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N13" t="str">
         <v>unknown</v>
       </c>
-      <c r="O4" t="str">
+      <c r="O13" t="str">
         <v>ગુજરાતી.</v>
       </c>
-      <c r="P4" t="str">
-        <v/>
-      </c>
-      <c r="Q4" t="str">
+      <c r="P13" t="str">
+        <v/>
+      </c>
+      <c r="Q13" t="str">
         <v>conv_0601kq9j10aff04bte8ak7gpqqbx</v>
       </c>
-      <c r="R4" t="str" xml:space="preserve">
+      <c r="R13" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -654,59 +1231,59 @@
 Agent: ધન્યવાદ. મા ઉમિયા અને વિશ્વ ઉમિયા ફાઉન્ડેશન વિશે સંક્ષિપ્ત સમાચાર સાંભળવા તમારી સા...</v>
       </c>
     </row>
-    <row r="5" xml:space="preserve">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
+    <row r="14" xml:space="preserve">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="str">
         <v>2026-04-28T08:04:48.175Z</v>
       </c>
-      <c r="C5" t="str">
-        <v/>
-      </c>
-      <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5" t="str">
-        <v/>
-      </c>
-      <c r="F5" t="str">
-        <v/>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
         <v>13</v>
       </c>
-      <c r="I5" t="str">
+      <c r="I14" t="str">
         <v>Hindi</v>
       </c>
-      <c r="J5" t="str">
+      <c r="J14" t="str">
         <v>hi</v>
       </c>
-      <c r="K5" t="str">
+      <c r="K14" t="str">
         <v>English, Gujarati, Hindi</v>
       </c>
-      <c r="L5" t="str">
+      <c r="L14" t="str">
         <v>Yes</v>
       </c>
-      <c r="M5" t="str">
+      <c r="M14" t="str">
         <v>Willing to join</v>
       </c>
-      <c r="N5" t="str">
+      <c r="N14" t="str">
         <v>willing_to_join</v>
       </c>
-      <c r="O5" t="str">
+      <c r="O14" t="str">
         <v>Okay. हाँ, मैं वही हूँ।</v>
       </c>
-      <c r="P5" t="str">
-        <v/>
-      </c>
-      <c r="Q5" t="str">
+      <c r="P14" t="str">
+        <v/>
+      </c>
+      <c r="Q14" t="str">
         <v>conv_9201kq9hsbc8egfs31f788amy56w</v>
       </c>
-      <c r="R5" t="str" xml:space="preserve">
+      <c r="R14" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -727,59 +1304,59 @@
 Agent: आपका स्वागत है।[grateful] माँ उमिया आपके और आपके परिवार के जीवन में शांति और सुख लाएं।[peaceful] आपका दिन शुभ हो।जय माँ उमिया 🙏</v>
       </c>
     </row>
-    <row r="6" xml:space="preserve">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
+    <row r="15" xml:space="preserve">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="str">
         <v>2026-04-28T08:02:30.875Z</v>
       </c>
-      <c r="C6" t="str">
-        <v/>
-      </c>
-      <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6" t="str">
-        <v/>
-      </c>
-      <c r="F6" t="str">
-        <v/>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6">
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
         <v>9</v>
       </c>
-      <c r="I6" t="str">
+      <c r="I15" t="str">
         <v>English</v>
       </c>
-      <c r="J6" t="str">
+      <c r="J15" t="str">
         <v>en</v>
       </c>
-      <c r="K6" t="str">
+      <c r="K15" t="str">
         <v>English, Gujarati, Hindi</v>
       </c>
-      <c r="L6" t="str">
+      <c r="L15" t="str">
         <v>Yes</v>
       </c>
-      <c r="M6" t="str">
+      <c r="M15" t="str">
         <v>Willing to join</v>
       </c>
-      <c r="N6" t="str">
+      <c r="N15" t="str">
         <v>willing_to_join</v>
       </c>
-      <c r="O6" t="str">
+      <c r="O15" t="str">
         <v>Okay. Sir.</v>
       </c>
-      <c r="P6" t="str">
-        <v/>
-      </c>
-      <c r="Q6" t="str">
+      <c r="P15" t="str">
+        <v/>
+      </c>
+      <c r="Q15" t="str">
         <v>conv_5901kq9hptgbe6rt4tjjqhnfmwk3</v>
       </c>
-      <c r="R6" t="str" xml:space="preserve">
+      <c r="R15" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be ...
@@ -793,115 +1370,115 @@
 Agent: सारा, महोदय। क्या आप माँ उमिया और विश्व उमिया फाउंडेशन के बारे में एक संक्षिप्त संदेश सुनने के लिए तैयार हैं?</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="str">
         <v>2026-04-28T06:42:54.419Z</v>
       </c>
-      <c r="C7" t="str">
-        <v/>
-      </c>
-      <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7" t="str">
-        <v/>
-      </c>
-      <c r="F7" t="str">
-        <v/>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="str">
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="str">
         <v>English</v>
       </c>
-      <c r="J7" t="str">
+      <c r="J16" t="str">
         <v>en</v>
       </c>
-      <c r="K7" t="str">
+      <c r="K16" t="str">
         <v>English</v>
       </c>
-      <c r="L7" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N7" t="str">
+      <c r="L16" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N16" t="str">
         <v>unknown</v>
       </c>
-      <c r="O7" t="str">
+      <c r="O16" t="str">
         <v>Transcript: Summary couldn't be generated for this call.</v>
       </c>
-      <c r="P7" t="str">
-        <v/>
-      </c>
-      <c r="Q7" t="str">
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
         <v>conv_7301kq9d735ve92stwtsszksq7v2</v>
       </c>
-      <c r="R7" t="str">
+      <c r="R16" t="str">
         <v>Transcript: Summary couldn't be generated for this call.</v>
       </c>
     </row>
-    <row r="8" xml:space="preserve">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
+    <row r="17" xml:space="preserve">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="str">
         <v>2026-04-28T06:42:53.484Z</v>
       </c>
-      <c r="C8" t="str">
-        <v/>
-      </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
-        <v/>
-      </c>
-      <c r="F8" t="str">
-        <v/>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8">
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
         <v>9</v>
       </c>
-      <c r="I8" t="str">
+      <c r="I17" t="str">
         <v>Gujarati</v>
       </c>
-      <c r="J8" t="str">
+      <c r="J17" t="str">
         <v>gu</v>
       </c>
-      <c r="K8" t="str">
+      <c r="K17" t="str">
         <v>English, Gujarati</v>
       </c>
-      <c r="L8" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M8" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N8" t="str">
+      <c r="L17" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N17" t="str">
         <v>unknown</v>
       </c>
-      <c r="O8" t="str">
+      <c r="O17" t="str">
         <v>હા</v>
       </c>
-      <c r="P8" t="str">
-        <v/>
-      </c>
-      <c r="Q8" t="str">
+      <c r="P17" t="str">
+        <v/>
+      </c>
+      <c r="Q17" t="str">
         <v>conv_9001kq9cx1bceky9cfvjzpq4tc09</v>
       </c>
-      <c r="R8" t="str" xml:space="preserve">
+      <c r="R17" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -918,62 +1495,62 @@
 Agent: ધન્યવાદ 🙏યુમિયા ધામ વિશ્વના સૌથી ઊંચા મંદિરોમાંના એક તરીકે વિકસાવવામાં આવી રહ્યું છે, જે આસ્થા, એકતા અને ભક્તિનું પ્રતીક છે.વિશ્વ ઉમિયા ફાઉન્ડેશન આધ્યાત્મિકતા, શિક્ષણ, સ્વાસ્...</v>
       </c>
     </row>
-    <row r="9" xml:space="preserve">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
+    <row r="18" xml:space="preserve">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="str">
         <v>2026-04-28T06:31:37.032Z</v>
       </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9" t="str">
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" t="str">
         <v>English</v>
       </c>
-      <c r="J9" t="str">
+      <c r="J18" t="str">
         <v>en</v>
       </c>
-      <c r="K9" t="str">
+      <c r="K18" t="str">
         <v>English</v>
       </c>
-      <c r="L9" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M9" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N9" t="str">
+      <c r="L18" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N18" t="str">
         <v>unknown</v>
       </c>
-      <c r="O9" t="str" xml:space="preserve">
+      <c r="O18" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
 Umiya Dham is being develope</v>
       </c>
-      <c r="P9" t="str">
-        <v/>
-      </c>
-      <c r="Q9" t="str">
+      <c r="P18" t="str">
+        <v/>
+      </c>
+      <c r="Q18" t="str">
         <v>conv_8301kq9chf18f59barx86mgyqn9a</v>
       </c>
-      <c r="R9" t="str" xml:space="preserve">
+      <c r="R18" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -981,121 +1558,121 @@
 At Vishv Umiya Foundation, the mission is to uplift society through ...</v>
       </c>
     </row>
-    <row r="10" xml:space="preserve">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
+    <row r="19" xml:space="preserve">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="str">
         <v>2026-04-28T06:30:38.685Z</v>
       </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10" t="str">
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19" t="str">
         <v>English</v>
       </c>
-      <c r="J10" t="str">
+      <c r="J19" t="str">
         <v>en</v>
       </c>
-      <c r="K10" t="str">
+      <c r="K19" t="str">
         <v>English</v>
       </c>
-      <c r="L10" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="M10" t="str">
-        <v>Unknown</v>
-      </c>
-      <c r="N10" t="str">
+      <c r="L19" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="N19" t="str">
         <v>unknown</v>
       </c>
-      <c r="O10" t="str" xml:space="preserve">
+      <c r="O19" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
 Umiya Dham is being develope</v>
       </c>
-      <c r="P10" t="str">
-        <v/>
-      </c>
-      <c r="Q10" t="str">
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
         <v>conv_6701kq9cg2eqer287bf4msmr1rhh</v>
       </c>
-      <c r="R10" t="str" xml:space="preserve">
+      <c r="R19" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
 Umiya Dham is being developed as one...</v>
       </c>
     </row>
-    <row r="11" xml:space="preserve">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
+    <row r="20" xml:space="preserve">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="str">
         <v>2026-04-28T05:38:40.915Z</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C20" t="str">
         <v>+919328481970</v>
       </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-      <c r="H11">
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
         <v>19</v>
       </c>
-      <c r="I11" t="str">
+      <c r="I20" t="str">
         <v>Hindi</v>
       </c>
-      <c r="J11" t="str">
+      <c r="J20" t="str">
         <v>hi</v>
       </c>
-      <c r="K11" t="str">
+      <c r="K20" t="str">
         <v>English, Hindi, Gujarati</v>
       </c>
-      <c r="L11" t="str">
+      <c r="L20" t="str">
         <v>Yes</v>
       </c>
-      <c r="M11" t="str">
+      <c r="M20" t="str">
         <v>Willing to join</v>
       </c>
-      <c r="N11" t="str">
+      <c r="N20" t="str">
         <v>willing_to_join</v>
       </c>
-      <c r="O11" t="str">
+      <c r="O20" t="str">
         <v>Okay, thank you.</v>
       </c>
-      <c r="P11" t="str">
+      <c r="P20" t="str">
         <v>CAd3fa254243c464a1730f45c7c56505ed</v>
       </c>
-      <c r="Q11" t="str">
+      <c r="Q20" t="str">
         <v>conv_5701kq99de98eg794mxra8d73bwb</v>
       </c>
-      <c r="R11" t="str" xml:space="preserve">
+      <c r="R20" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -1122,59 +1699,59 @@
 Agent: ...</v>
       </c>
     </row>
-    <row r="12" xml:space="preserve">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
+    <row r="21" xml:space="preserve">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="str">
         <v>2026-04-28T05:28:57.765Z</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C21" t="str">
         <v>+919328481970</v>
       </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-      <c r="H12">
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
         <v>15</v>
       </c>
-      <c r="I12" t="str">
+      <c r="I21" t="str">
         <v>Hindi</v>
       </c>
-      <c r="J12" t="str">
+      <c r="J21" t="str">
         <v>hi</v>
       </c>
-      <c r="K12" t="str">
+      <c r="K21" t="str">
         <v>English, Hindi</v>
       </c>
-      <c r="L12" t="str">
+      <c r="L21" t="str">
         <v>Yes</v>
       </c>
-      <c r="M12" t="str">
+      <c r="M21" t="str">
         <v>Willing to join</v>
       </c>
-      <c r="N12" t="str">
+      <c r="N21" t="str">
         <v>willing_to_join</v>
       </c>
-      <c r="O12" t="str">
+      <c r="O21" t="str">
         <v>Yes, जानना चाहूँगा।</v>
       </c>
-      <c r="P12" t="str">
+      <c r="P21" t="str">
         <v>CA34c672f4a33b63610704a7d7f3ade6ab</v>
       </c>
-      <c r="Q12" t="str">
+      <c r="Q21" t="str">
         <v>conv_8201kq98we89eh6v5hpy42ncxkfd</v>
       </c>
-      <c r="R12" t="str" xml:space="preserve">
+      <c r="R21" t="str" xml:space="preserve">
         <v xml:space="preserve">Agent: Namaste 
 I am calling from Vishv Umiya Foundation. Which language are you comfortable speaking — English, Hindi, or Gujarati?
 Would you be willing to hear a brief message about Maa Umiya and our mission?
@@ -1198,7 +1775,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>